<commit_message>
Autofix policy: what Claude fixes itself, what it escalates
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013mm46m7T8HwJboSANTcNw4
</commit_message>
<xml_diff>
--- a/marketing/Education_Groups_Target_Directory.xlsx
+++ b/marketing/Education_Groups_Target_Directory.xlsx
@@ -7890,7 +7890,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <tabColor rgb="FFF2B705"/>
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:H45"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -8615,7 +8615,7 @@
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -34479,7 +34479,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <tabColor rgb="FF9B1C1C"/>
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:D33"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -34956,7 +34956,7 @@
   <autoFilter ref="A1:D33"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>